<commit_message>
feat: major UI/UX and logic improvements
- Разделение js/collections/main.js на модули (core, render, modals, schools)
- Исправлено закрытие модалок при выделении текста (отключён клик по фону)
- Занятия: новая логика автоподстановки тем по фиксированному расписанию (кнопка 'Темы автоматически')
- Сборы: добавлены статусы, кнопки 'Закрепить'/'Открепить', мгновенное обновление статусов в модалке
- Сводная ведомость: подстановка руководителя школы (тег {{HEAD_TEACHER}}), границы, нумерация
- Временный журнал: вертикальные столбцы итоговых оценок по предметам (теги {{FINAL_...}})
- Оценки: фильтр 'Все школы', режим 'Все предметы', индикатор загрузки, горизонтальная прокрутка
- Взвода: удалена кнопка 'Сформировать документ', дублирование кнопки 'Добавить во взвод'
- Документы: карточки документов с описанием и редактированием
- Тёмная тема: исправлены поля ввода, поиск, textarea
</commit_message>
<xml_diff>
--- a/templates/contracts/svodnaya_template.xlsx
+++ b/templates/contracts/svodnaya_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\templates\contracts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\centrcom\templates\contracts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FEC9241-A12C-4D2E-9B22-01B6FE998F3A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2250DB-49A8-49FC-BE5E-3BDC1C998BCC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="26730" windowHeight="20715" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -81,24 +81,6 @@
     <t>{{ROWS}}</t>
   </si>
   <si>
-    <t>Представитель учебной организации_______________________________________________________В.Н.Литвиненко</t>
-  </si>
-  <si>
-    <t>Представитель воинской части (соединения)__________________________________________________________</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> м.п.</t>
-  </si>
-  <si>
-    <t>Генеральный директор ООО «Центр +»</t>
-  </si>
-  <si>
-    <t>К. К. Ляхов</t>
-  </si>
-  <si>
-    <t xml:space="preserve">                                                                                 м.п.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Выбор места для стрельбы, </t>
   </si>
   <si>
@@ -214,6 +196,24 @@
   </si>
   <si>
     <t>{{FINAL_OVERALL}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                                м.п.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                                                                                               м.п.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Представитель учебной организации                 ___________________________________________________ </t>
+  </si>
+  <si>
+    <t>{{HEAD_TEACHER}}</t>
+  </si>
+  <si>
+    <t>Представитель воинской части (соединения)    ___________________________________________________</t>
+  </si>
+  <si>
+    <t>Генеральный директор ООО «Центр +»            ____________________________________________________     К. К. Ляхов</t>
   </si>
 </sst>
 </file>
@@ -394,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -415,6 +415,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" textRotation="90" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -728,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA15"/>
+  <dimension ref="A1:AA17"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.28515625" style="3" customWidth="1"/>
@@ -742,7 +746,8 @@
     <col min="24" max="24" width="4.5703125" style="3" customWidth="1"/>
     <col min="25" max="26" width="4.7109375" style="3" customWidth="1"/>
     <col min="27" max="27" width="5.5703125" style="3" customWidth="1"/>
-    <col min="28" max="16384" width="9.140625" style="1"/>
+    <col min="28" max="28" width="9.140625" style="1" customWidth="1"/>
+    <col min="29" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -836,107 +841,107 @@
       <c r="AA3" s="1"/>
     </row>
     <row r="5" spans="1:27" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="8" t="s">
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="8" t="s">
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="8" t="s">
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="10"/>
-      <c r="T5" s="8" t="s">
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="12"/>
+      <c r="T5" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="U5" s="9"/>
-      <c r="V5" s="10"/>
-      <c r="W5" s="8" t="s">
+      <c r="U5" s="11"/>
+      <c r="V5" s="12"/>
+      <c r="W5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="X5" s="9"/>
-      <c r="Y5" s="9"/>
-      <c r="Z5" s="10"/>
-      <c r="AA5" s="14" t="s">
+      <c r="X5" s="11"/>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="12"/>
+      <c r="AA5" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="12"/>
-      <c r="N6" s="12"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
-      <c r="S6" s="13"/>
-      <c r="T6" s="11"/>
-      <c r="U6" s="12"/>
-      <c r="V6" s="13"/>
-      <c r="W6" s="11"/>
-      <c r="X6" s="12"/>
-      <c r="Y6" s="12"/>
-      <c r="Z6" s="13"/>
-      <c r="AA6" s="15"/>
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="13"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="15"/>
+      <c r="W6" s="13"/>
+      <c r="X6" s="14"/>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="15"/>
+      <c r="AA6" s="17"/>
     </row>
     <row r="7" spans="1:27" ht="206.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
       <c r="C7" s="5" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>10</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>11</v>
@@ -951,40 +956,40 @@
         <v>14</v>
       </c>
       <c r="O7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="R7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="S7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="T7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="P7" s="5" t="s">
+      <c r="U7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="V7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="Q7" s="5" t="s">
+      <c r="Y7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="R7" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="S7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="T7" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="U7" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="V7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="X7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="Y7" s="5" t="s">
-        <v>37</v>
-      </c>
       <c r="Z7" s="7" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="AA7" s="4"/>
     </row>
@@ -1071,113 +1076,240 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" ht="94.5" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="J9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="K9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="L9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="M9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="N9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="O9" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J9" s="3" t="s">
+      <c r="P9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="Q9" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="R9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="S9" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="N9" s="3" t="s">
+      <c r="T9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="O9" s="3" t="s">
+      <c r="U9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="P9" s="3" t="s">
+      <c r="V9" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="Q9" s="3" t="s">
+      <c r="W9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="R9" s="3" t="s">
+      <c r="X9" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="S9" s="3" t="s">
+      <c r="Y9" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="T9" s="3" t="s">
+      <c r="Z9" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="U9" s="3" t="s">
+      <c r="AA9" s="8" t="s">
         <v>56</v>
-      </c>
-      <c r="V9" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="W9" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="X9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y9" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="Z9" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA9" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="A13" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="9"/>
+      <c r="S13" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="U13" s="9"/>
+      <c r="V13" s="9"/>
+      <c r="W13" s="9"/>
+      <c r="X13" s="9"/>
+      <c r="Y13" s="9"/>
+      <c r="Z13" s="9"/>
+      <c r="AA13" s="9"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>22</v>
-      </c>
+      <c r="A14" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
+      <c r="P14" s="9"/>
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9"/>
+      <c r="S14" s="9"/>
+      <c r="T14" s="9"/>
+      <c r="U14" s="9"/>
+      <c r="V14" s="9"/>
+      <c r="W14" s="9"/>
+      <c r="X14" s="9"/>
+      <c r="Y14" s="9"/>
+      <c r="Z14" s="9"/>
+      <c r="AA14" s="9"/>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>23</v>
-      </c>
+      <c r="A15" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="9"/>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9"/>
+      <c r="S15" s="9"/>
+      <c r="T15" s="9"/>
+      <c r="U15" s="9"/>
+      <c r="V15" s="9"/>
+      <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+      <c r="Y15" s="9"/>
+      <c r="Z15" s="9"/>
+      <c r="AA15" s="9"/>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+      <c r="S16" s="9"/>
+      <c r="T16" s="9"/>
+      <c r="U16" s="9"/>
+      <c r="V16" s="9"/>
+      <c r="W16" s="9"/>
+      <c r="X16" s="9"/>
+      <c r="Y16" s="9"/>
+      <c r="Z16" s="9"/>
+      <c r="AA16" s="9"/>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="9"/>
+      <c r="T17" s="9"/>
+      <c r="U17" s="9"/>
+      <c r="V17" s="9"/>
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
+      <c r="Y17" s="9"/>
+      <c r="Z17" s="9"/>
+      <c r="AA17" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>